<commit_message>
Housekeeping - Update data - Add/update tests
</commit_message>
<xml_diff>
--- a/inst/extdata/mitigations.xlsx
+++ b/inst/extdata/mitigations.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="26">
   <si>
     <t xml:space="preserve">You must supply start and end nodes</t>
   </si>
@@ -48,16 +48,10 @@
     <t xml:space="preserve">end_node</t>
   </si>
   <si>
-    <t xml:space="preserve">short_en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">long_en</t>
-  </si>
-  <si>
-    <t xml:space="preserve">short_fr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">long_fr</t>
+    <t xml:space="preserve">short</t>
+  </si>
+  <si>
+    <t xml:space="preserve">long</t>
   </si>
   <si>
     <t xml:space="preserve">Marine Birds</t>
@@ -69,9 +63,6 @@
     <t xml:space="preserve">By working selectively, avoid direct problems.</t>
   </si>
   <si>
-    <t xml:space="preserve">frenchxx</t>
-  </si>
-  <si>
     <t xml:space="preserve">Relocate</t>
   </si>
   <si>
@@ -106,9 +97,6 @@
   </si>
   <si>
     <t xml:space="preserve">Create Habitat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Créer des habitats</t>
   </si>
   <si>
     <t xml:space="preserve">Option 5</t>
@@ -206,7 +194,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -225,10 +213,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -384,12 +368,12 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -437,16 +421,12 @@
       <c r="E1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>2</v>
@@ -455,18 +435,15 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>3</v>
@@ -475,18 +452,15 @@
         <v>5</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2</v>
@@ -495,205 +469,202 @@
         <v>4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -734,341 +705,337 @@
       <c r="E1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1109,221 +1076,217 @@
       <c r="E1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1364,16 +1327,12 @@
       <c r="E1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>2</v>
@@ -1382,18 +1341,16 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>3</v>
@@ -1402,18 +1359,16 @@
         <v>5</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="F3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>6</v>
@@ -1422,18 +1377,16 @@
         <v>88</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="F4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>48</v>
@@ -1442,18 +1395,16 @@
         <v>88</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="F5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>47</v>
@@ -1462,16 +1413,14 @@
         <v>50</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="F6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>47</v>
@@ -1480,16 +1429,14 @@
         <v>52</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E7" s="2"/>
-      <c r="F7" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>14</v>
@@ -1498,16 +1445,14 @@
         <v>33</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>15</v>
@@ -1516,16 +1461,14 @@
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E9" s="2"/>
-      <c r="F9" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>13</v>
@@ -1534,16 +1477,14 @@
         <v>22</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E10" s="2"/>
-      <c r="F10" s="4" t="s">
-        <v>26</v>
-      </c>
+      <c r="F10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>2</v>
@@ -1552,16 +1493,14 @@
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E11" s="2"/>
-      <c r="F11" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="F11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>3</v>
@@ -1570,16 +1509,14 @@
         <v>13</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E12" s="2"/>
-      <c r="F12" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="F12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>3</v>
@@ -1588,16 +1525,14 @@
         <v>14</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E13" s="2"/>
-      <c r="F13" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="F13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1607,262 +1542,262 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1887,12 +1822,12 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="12.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="11.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="10.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="5" width="9.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="5" width="9.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="5" width="8.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1911,301 +1846,297 @@
       <c r="E1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>